<commit_message>
Raw vs Clean metrics: label reconciliation, issue counts, whale impact, leakage diagnostic; cleaning script drops leakage/identifier columns
</commit_message>
<xml_diff>
--- a/TW1_Audit_Findings.xlsx
+++ b/TW1_Audit_Findings.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>5.4% vs 4.9%</t>
+          <t>5.8% vs 4.9%</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>21.4</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="60">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>unique_customers</t>
+          <t>ambiguous_label_rows_excluded</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2500</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61">
@@ -1384,11 +1384,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>churn_2022_share_all_pct</t>
+          <t>unique_customers</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>5.8</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="62">
@@ -1399,11 +1399,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>churn_2023_share_all_pct</t>
+          <t>churn_2022_share_all_pct</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>13.8</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="63">
@@ -1414,13 +1414,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>largest_industry</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
+          <t>churn_2023_share_all_pct</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>13.8</v>
       </c>
     </row>
     <row r="64">
@@ -1431,11 +1429,13 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>largest_industry_share_pct</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>17.8</v>
+          <t>largest_industry</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -1446,13 +1446,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>highest_churn_industry</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
+          <t>largest_industry_share_pct</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>17.8</v>
       </c>
     </row>
     <row r="66">
@@ -1463,11 +1461,13 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>highest_churn_industry_rate_pct</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>24.2</v>
+          <t>highest_churn_industry</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -1478,13 +1478,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>highest_churn_contract</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Month-to-Month</t>
-        </is>
+          <t>highest_churn_industry_rate_pct</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>22.4</v>
       </c>
     </row>
     <row r="68">
@@ -1495,11 +1493,13 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>highest_churn_contract_rate_pct</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>33.7</v>
+          <t>highest_churn_contract</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Month-to-Month</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -1510,13 +1510,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>lowest_churn_contract</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>2 Year</t>
-        </is>
+          <t>highest_churn_contract_rate_pct</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>32.2</v>
       </c>
     </row>
     <row r="70">
@@ -1527,11 +1525,13 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>lowest_churn_contract_rate_pct</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>15.3</v>
+          <t>lowest_churn_contract</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -1542,11 +1542,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>leakage_churn_yes_with_date</t>
+          <t>lowest_churn_contract_rate_pct</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>491</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="72">
@@ -1557,11 +1557,86 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
+          <t>leakage_churn_yes_with_date</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>part2_3</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>leakage_churn_yes_total</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>part2_3</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>leakage_churn_no_with_date</t>
         </is>
       </c>
-      <c r="C72" t="n">
+      <c r="C74" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>part2_3</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>leakage_churn_no_total</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>part2_3</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>leakage_ambiguous_with_date</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>part2_3</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>leakage_ambiguous_total</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -23999,7 +24074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -24027,104 +24102,117 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>1 (ambiguous)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.951</v>
+        <v>0.98</v>
       </c>
       <c r="C2" t="n">
-        <v>0.049</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.946</v>
+        <v>0.951</v>
       </c>
       <c r="C3" t="n">
-        <v>0.054</v>
+        <v>0.049</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.95</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.931</v>
+        <v>0.95</v>
       </c>
       <c r="C5" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.964</v>
+        <v>0.931</v>
       </c>
       <c r="C6" t="n">
-        <v>0.036</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.948</v>
+        <v>0.964</v>
       </c>
       <c r="C7" t="n">
-        <v>0.052</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.953</v>
+        <v>0.948</v>
       </c>
       <c r="C8" t="n">
-        <v>0.047</v>
+        <v>0.052</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.047</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Tech</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>0.954</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C10" t="n">
         <v>0.046</v>
       </c>
     </row>
@@ -24262,10 +24350,10 @@
         <v>445</v>
       </c>
       <c r="C2" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="D2" t="n">
-        <v>20.2</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="3">
@@ -24278,10 +24366,10 @@
         <v>443</v>
       </c>
       <c r="C3" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D3" t="n">
-        <v>21.4</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="4">
@@ -24294,10 +24382,10 @@
         <v>414</v>
       </c>
       <c r="C4" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D4" t="n">
-        <v>19.1</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="5">
@@ -24310,10 +24398,10 @@
         <v>409</v>
       </c>
       <c r="C5" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D5" t="n">
-        <v>21.3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -24326,10 +24414,10 @@
         <v>401</v>
       </c>
       <c r="C6" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D6" t="n">
-        <v>24.2</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="7">
@@ -24342,10 +24430,10 @@
         <v>388</v>
       </c>
       <c r="C7" t="n">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="D7" t="n">
-        <v>22.2</v>
+        <v>19.1</v>
       </c>
     </row>
   </sheetData>
@@ -25230,10 +25318,10 @@
         <v>817</v>
       </c>
       <c r="C2" t="n">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="D2" t="n">
-        <v>33.7</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="3">
@@ -25255,33 +25343,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1 Year</t>
+          <t>2 Year</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>820</v>
+        <v>813</v>
       </c>
       <c r="C4" t="n">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="D4" t="n">
-        <v>15.5</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2 Year</t>
+          <t>1 Year</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="C5" t="n">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="D5" t="n">
-        <v>15.3</v>
+        <v>12.9</v>
       </c>
     </row>
   </sheetData>
@@ -25339,13 +25427,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18.5</v>
+        <v>16.6</v>
       </c>
       <c r="C2" t="n">
-        <v>19.5</v>
+        <v>18.7</v>
       </c>
       <c r="D2" t="n">
-        <v>36.6</v>
+        <v>34.1</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -25358,13 +25446,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18.9</v>
+        <v>14.8</v>
       </c>
       <c r="C3" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>32.3</v>
+        <v>29.9</v>
       </c>
       <c r="E3" t="n">
         <v>12.5</v>
@@ -25377,13 +25465,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.5</v>
+        <v>6.1</v>
       </c>
       <c r="C4" t="n">
-        <v>13.2</v>
+        <v>9.9</v>
       </c>
       <c r="D4" t="n">
-        <v>37</v>
+        <v>36.3</v>
       </c>
       <c r="E4" t="n">
         <v>18.2</v>
@@ -25396,13 +25484,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.8</v>
+        <v>11.2</v>
       </c>
       <c r="C5" t="n">
-        <v>14.8</v>
+        <v>12.3</v>
       </c>
       <c r="D5" t="n">
-        <v>35.1</v>
+        <v>34.4</v>
       </c>
       <c r="E5" t="n">
         <v>25</v>
@@ -25415,13 +25503,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.5</v>
+        <v>14.4</v>
       </c>
       <c r="C6" t="n">
-        <v>14.9</v>
+        <v>12.8</v>
       </c>
       <c r="D6" t="n">
-        <v>28.4</v>
+        <v>26.2</v>
       </c>
       <c r="E6" t="n">
         <v>10</v>
@@ -25434,13 +25522,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17.1</v>
+        <v>14.7</v>
       </c>
       <c r="C7" t="n">
-        <v>13.3</v>
+        <v>12.6</v>
       </c>
       <c r="D7" t="n">
-        <v>32.9</v>
+        <v>32.1</v>
       </c>
       <c r="E7" t="n">
         <v>20</v>
@@ -25457,10 +25545,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
@@ -25485,27 +25573,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>1 (ambiguous)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1966</v>
+        <v>43</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>43</v>
+        <v>1966</v>
       </c>
       <c r="C3" t="n">
-        <v>491</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>